<commit_message>
added cenrter create validation in it and bulkuploading changes
</commit_message>
<xml_diff>
--- a/public/samples/voucher_sample.xlsx
+++ b/public/samples/voucher_sample.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
   <si>
     <t>voucher_code</t>
   </si>
@@ -27,6 +27,15 @@
     <t>purchase_date</t>
   </si>
   <si>
+    <t>course_category</t>
+  </si>
+  <si>
+    <t>course_code</t>
+  </si>
+  <si>
+    <t>course_name</t>
+  </si>
+  <si>
     <t>expiry_date</t>
   </si>
   <si>
@@ -34,6 +43,72 @@
   </si>
   <si>
     <t>cost</t>
+  </si>
+  <si>
+    <t>VCH001</t>
+  </si>
+  <si>
+    <t>Sunrise Traders</t>
+  </si>
+  <si>
+    <t>Cloud Computing</t>
+  </si>
+  <si>
+    <t>AWS01</t>
+  </si>
+  <si>
+    <t>AWS</t>
+  </si>
+  <si>
+    <t>VCH002</t>
+  </si>
+  <si>
+    <t>Bright Distribution Co.</t>
+  </si>
+  <si>
+    <t>AZUR01</t>
+  </si>
+  <si>
+    <t>Azur</t>
+  </si>
+  <si>
+    <t>VCH003</t>
+  </si>
+  <si>
+    <t>Global Supplies</t>
+  </si>
+  <si>
+    <t>GoogleCloud01</t>
+  </si>
+  <si>
+    <t>Google Cloud</t>
+  </si>
+  <si>
+    <t>VCH004</t>
+  </si>
+  <si>
+    <t>Tech Solutions Pvt. Ltd.</t>
+  </si>
+  <si>
+    <t>Digital Marketing</t>
+  </si>
+  <si>
+    <t>DM01</t>
+  </si>
+  <si>
+    <t>Digital Marketing Professional</t>
+  </si>
+  <si>
+    <t>VCH005</t>
+  </si>
+  <si>
+    <t>Information Technology (IT)</t>
+  </si>
+  <si>
+    <t>DI01</t>
+  </si>
+  <si>
+    <t>Diploma in Information Technology</t>
   </si>
 </sst>
 </file>
@@ -79,14 +154,14 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -389,71 +464,186 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultColWidth="16.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46235</v>
+      </c>
+      <c r="G2" s="2">
+        <v>46600</v>
+      </c>
+      <c r="H2" s="1">
+        <v>1000</v>
+      </c>
+      <c r="I2" s="1">
+        <v>850</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
+    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46239</v>
+      </c>
+      <c r="G3" s="2">
+        <v>46604</v>
+      </c>
+      <c r="H3" s="1">
+        <v>1200</v>
+      </c>
+      <c r="I3" s="1">
+        <v>1000</v>
+      </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
+    <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46244</v>
+      </c>
+      <c r="G4" s="2">
+        <v>46609</v>
+      </c>
+      <c r="H4" s="1">
+        <v>1500</v>
+      </c>
+      <c r="I4" s="1">
+        <v>1300</v>
+      </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
+    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46249</v>
+      </c>
+      <c r="G5" s="2">
+        <v>46614</v>
+      </c>
+      <c r="H5" s="1">
+        <v>900</v>
+      </c>
+      <c r="I5" s="1">
+        <v>750</v>
+      </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
+    <row r="6" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46254</v>
+      </c>
+      <c r="G6" s="2">
+        <v>46619</v>
+      </c>
+      <c r="H6" s="1">
+        <v>2000</v>
+      </c>
+      <c r="I6" s="1">
+        <v>1750</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="0" copies="0" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
shown proper data in excel as a sample
</commit_message>
<xml_diff>
--- a/public/samples/voucher_sample.xlsx
+++ b/public/samples/voucher_sample.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>voucher_code</t>
   </si>
@@ -58,57 +58,6 @@
   </si>
   <si>
     <t>AWS</t>
-  </si>
-  <si>
-    <t>VCH002</t>
-  </si>
-  <si>
-    <t>Bright Distribution Co.</t>
-  </si>
-  <si>
-    <t>AZUR01</t>
-  </si>
-  <si>
-    <t>Azur</t>
-  </si>
-  <si>
-    <t>VCH003</t>
-  </si>
-  <si>
-    <t>Global Supplies</t>
-  </si>
-  <si>
-    <t>GoogleCloud01</t>
-  </si>
-  <si>
-    <t>Google Cloud</t>
-  </si>
-  <si>
-    <t>VCH004</t>
-  </si>
-  <si>
-    <t>Tech Solutions Pvt. Ltd.</t>
-  </si>
-  <si>
-    <t>Digital Marketing</t>
-  </si>
-  <si>
-    <t>DM01</t>
-  </si>
-  <si>
-    <t>Digital Marketing Professional</t>
-  </si>
-  <si>
-    <t>VCH005</t>
-  </si>
-  <si>
-    <t>Information Technology (IT)</t>
-  </si>
-  <si>
-    <t>DI01</t>
-  </si>
-  <si>
-    <t>Diploma in Information Technology</t>
   </si>
 </sst>
 </file>
@@ -465,7 +414,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultColWidth="16.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="51.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.5703125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
@@ -496,7 +456,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -525,121 +485,49 @@
         <v>850</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46239</v>
-      </c>
-      <c r="G3" s="2">
-        <v>46604</v>
-      </c>
-      <c r="H3" s="1">
-        <v>1200</v>
-      </c>
-      <c r="I3" s="1">
-        <v>1000</v>
-      </c>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
     </row>
-    <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46244</v>
-      </c>
-      <c r="G4" s="2">
-        <v>46609</v>
-      </c>
-      <c r="H4" s="1">
-        <v>1500</v>
-      </c>
-      <c r="I4" s="1">
-        <v>1300</v>
-      </c>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
     </row>
-    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46249</v>
-      </c>
-      <c r="G5" s="2">
-        <v>46614</v>
-      </c>
-      <c r="H5" s="1">
-        <v>900</v>
-      </c>
-      <c r="I5" s="1">
-        <v>750</v>
-      </c>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
     </row>
-    <row r="6" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46254</v>
-      </c>
-      <c r="G6" s="2">
-        <v>46619</v>
-      </c>
-      <c r="H6" s="1">
-        <v>2000</v>
-      </c>
-      <c r="I6" s="1">
-        <v>1750</v>
-      </c>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>